<commit_message>
Added Ex4A file and updated kabakibi_Ex3A_tables file
</commit_message>
<xml_diff>
--- a/Kabakibi_Ex3A_tables.xlsx
+++ b/Kabakibi_Ex3A_tables.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6350" firstSheet="1" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6350" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Owner" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="37">
   <si>
     <t>owner_id</t>
   </si>
@@ -94,16 +94,69 @@
   </si>
   <si>
     <t>status</t>
+  </si>
+  <si>
+    <t>Jane</t>
+  </si>
+  <si>
+    <t>Bella</t>
+  </si>
+  <si>
+    <t>Havanese</t>
+  </si>
+  <si>
+    <t>11 lbs (Small)</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>https://t3.ftcdn.net/jpg/03/58/32/92/360_F_358329259_MWxTVvYonW8L1qxUgNn90uWN4Yh0atZn.jpg</t>
+  </si>
+  <si>
+    <t>2 Years</t>
+  </si>
+  <si>
+    <t>Steve</t>
+  </si>
+  <si>
+    <t>Mary Smith, 5550198888</t>
+  </si>
+  <si>
+    <t>09:00 AM - 10:00 AM</t>
+  </si>
+  <si>
+    <t>https://maps.walktrack.com/path/1012</t>
+  </si>
+  <si>
+    <t>Fresh water provided after the walk. Locked the back door.</t>
+  </si>
+  <si>
+    <t>Credit Card</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>521 street ave, Newark NJ 07102</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -138,15 +191,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -425,10 +482,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -445,6 +503,20 @@
         <v>3</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>101</v>
+      </c>
+      <c r="B2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2">
+        <v>2223334444</v>
+      </c>
+      <c r="D2" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -452,11 +524,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
@@ -485,14 +558,43 @@
         <v>9</v>
       </c>
     </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>101</v>
+      </c>
+      <c r="C2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="13.90625" bestFit="1" customWidth="1"/>
@@ -513,6 +615,20 @@
         <v>11</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>402</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2">
+        <v>2224445555</v>
+      </c>
+      <c r="D2" t="s">
+        <v>30</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -520,12 +636,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="8.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="34.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -551,19 +668,46 @@
         <v>16</v>
       </c>
     </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1012</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>402</v>
+      </c>
+      <c r="D2" s="4">
+        <v>46130</v>
+      </c>
+      <c r="E2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.7265625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.81640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -586,6 +730,26 @@
         <v>21</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>5001</v>
+      </c>
+      <c r="B2">
+        <v>1012</v>
+      </c>
+      <c r="C2">
+        <v>35</v>
+      </c>
+      <c r="D2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" s="4">
+        <v>46130</v>
+      </c>
+      <c r="F2" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>